<commit_message>
Nesta aula contunuamos com a parte de bibliotecas  e comecamos um exercicio
</commit_message>
<xml_diff>
--- a/aula12/cadastro_alunos.xlsx
+++ b/aula12/cadastro_alunos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,125 +432,19 @@
           <t>altura</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>israel</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="F1" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>rafael</t>
-        </is>
-      </c>
-      <c r="H1" t="n">
-        <v>1.88</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>israel</t>
+          <t>Girassol</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="C2" t="n">
         <v>1.7</v>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>na</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>israel</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>rafael</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>1.88</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>israel</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>25</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1.87</v>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>israel</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>25</v>
-      </c>
-      <c r="C6" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>